<commit_message>
增加"dev": "vite --host 0.0.0.0 --port 8080",
</commit_message>
<xml_diff>
--- a/data/projects/70e5ca737ae5433e9f0f3134d216acf7/早期介入/交付预案/输出结果/智算部件配置信息表.xlsx
+++ b/data/projects/70e5ca737ae5433e9f0f3134d216acf7/早期介入/交付预案/输出结果/智算部件配置信息表.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,6 +496,33 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>V2.3_20260614220356_DRB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>V2.3_20260614220356_DRB</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>V2.3_20260614220356_DRB</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
merge remote feature_new and preserve local proposal updates
Pull latest fork/feature_new into local branch, then reapply local proposal and data artifact changes with conflict resolution favoring local regenerated outputs to keep workspace continuity.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/projects/70e5ca737ae5433e9f0f3134d216acf7/早期介入/交付预案/输出结果/智算部件配置信息表.xlsx
+++ b/data/projects/70e5ca737ae5433e9f0f3134d216acf7/早期介入/交付预案/输出结果/智算部件配置信息表.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -523,6 +523,33 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>V2.4_20260615171738_DRB</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>V2.4_20260615171738_DRB</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>V2.4_20260615171738_DRB</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>